<commit_message>
Update Selections worksheet with offer note
</commit_message>
<xml_diff>
--- a/files/Prephase-Selections-Worksheet.xlsx
+++ b/files/Prephase-Selections-Worksheet.xlsx
@@ -1257,17 +1257,17 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
         <v>20</v>
       </c>

</xml_diff>